<commit_message>
improved plot size class ranges
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/geographical_feature/node_metrics_paper.xlsx
+++ b/southern_europe/italy_data/geographical_feature/node_metrics_paper.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nodes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="truck" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="railway" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw_data" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="readme" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="truck_availability" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="nodes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="truck" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="pipeline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="railway" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="raw_data" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="readme" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="truck_availability" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="paper_names" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'nodes'!$H$1:$H$48</definedName>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Aptos Narrow"/>
       <color theme="1"/>
@@ -133,6 +134,9 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -194,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -237,6 +241,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -41942,4 +41947,1302 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>node_id</t>
+        </is>
+      </c>
+      <c r="B1" s="40" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="C1" s="40" t="inlineStr">
+        <is>
+          <t>node_type</t>
+        </is>
+      </c>
+      <c r="D1" s="40" t="inlineStr">
+        <is>
+          <t>paper_name</t>
+        </is>
+      </c>
+      <c r="E1" s="40" t="inlineStr">
+        <is>
+          <t>sector_in_paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TRM - TERMOVALORIZZATORE DEL GERBIDO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Torino WtE plant</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ROBILANTE cement plant</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Robilante cement plant</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Trino Vercellese</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Trino Vercellese rail terminal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Colacem - Stabilimento di Caravate</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Caravate cement plant</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Holcim (Italia) S.p.A.-unità produttiva di Ternate</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ternate cement plant</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE BUSTO ARSIZIO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Busto Arsizio WtE plant</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RAFFINERIA SARPOM DI TRECATE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Refining</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Trecate refinery</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Refining</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LOMELLINA ENERGIA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Parona WtE plant</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RAFFINERIA DI SANNAZZARO DE' BURGONDI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Refining</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sannazzaro de' Burgondi refinery</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Refining</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Iplom S.p.A - Raffineria di Busalla</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Refining</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Busalla refinery</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Refining</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE COMO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Como WtE plant</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE DI DESIO</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Desio WtE plant</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SILLA 2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Milano WtE plant</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TermoTrezzo</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Trezzo sull'Adda WtE plant</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Segrate</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Segrate rail terminal</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE DI CORTEOLONA E GENZONE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Corteolona WtE plant</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Impianto di termovalorizzazione di Valmadrera</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Valmadrera WtE plant</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Italcementi Calusco D'Adda</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Calusco d'Adda cement plant</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Termovalorizzatore di Dalmine</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Dalmine WtE plant</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Piacenza</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Piacenza WtE plant</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Piacenza</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Piacenza cement plant</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VERNASCA cement plant</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Vernasca cement plant</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Stabilimento di Tavernola Bergamasca</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Tavernola Bergamasca cement plant</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE DI BRESCIA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Brescia WtE plant</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Italcementi di Rezzato</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Rezzato cement plant</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE - PAIP</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Parma WtE plant</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZAOTRE DI VERONA</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Verona WtE plant</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HERAMBIENTE S.R.L.  - Termovalorizzatore</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Modena WtE plant</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TERMOVALORIZZATORE DI BOLZANO</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Bolzano WtE plant</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ferrara</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ferrara WtE plant</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Ferrara</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FertilizersCombustion</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Ferrara fertiliser plant (combustion)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Fertilisers</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ferrara</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FertilizersSMR</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ferrara fertiliser plant (SMR)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Fertilisers</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>FRULLO ENERGIA AMBIENTE S.R.L.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Granarolo dell'Emilia WtE plant</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MONSELICE cement plant</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Monselice cement plant</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Fassa Cerano Dolce</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Dolcè lime plant</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cementirossi - Cementeria di Pederobba</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pederobba cement plant</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Impianto di Termovalorizzazione di San Lazzaro (PD)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Padova WtE plant</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HERAMBIENTE - 3^ LINEA</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Forlì WtE plant</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>STABILIMENTO DI PONTE DELLA PRIULA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Susegana cement plant</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Ravenna</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ravenna industrial cluster</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Venezia Marghera Scalo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Venezia Marghera rail terminal</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>FANNA cement plant</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Fanna cement plant</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Termovalorizzatore di Rimini</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Rimini WtE plant</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Impianto di Termovalorizzazione Rifiuti di Trieste</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Trieste WtE plant</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>WtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Eni S.p.A Casalborsetti</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Casalborsetti onshore terminal</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Porto Corsini</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Porto Corsini offshore storage</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Modena-H</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Modena transport hub</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Unicalce Val Brembilla Lime</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Val Brembilla lime plant</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Fassa Montichiari Lime</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Montichiari lime plant</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Unicalce Bernezzo</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Bernezzo lime plant</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>